<commit_message>
Begin tech KT session content creation, clean up
</commit_message>
<xml_diff>
--- a/KT_Session_Question_Review/00_Drafts/SHRSS_KT_Session_Questions_Analysis_Expanded_v3.xlsx
+++ b/KT_Session_Question_Review/00_Drafts/SHRSS_KT_Session_Questions_Analysis_Expanded_v3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lambert/Documents/Projects/SHRSS/SHRSS_Knowledge_Transfer/KT_Session_Question_Analysis/00_Drafts/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lambert/Documents/Projects/SHRSS/SHRSS_Knowledge_Transfer/KT_Session_Question_Review/00_Drafts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBCC1F2-AEF8-0F42-B6E0-1C7CDC2B5666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8BCADE0-086A-ED4A-B525-80AC426CD357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1640" yWindow="760" windowWidth="32920" windowHeight="20020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1640" yWindow="760" windowWidth="32920" windowHeight="20020" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jobs" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="560">
   <si>
     <t>Question</t>
   </si>
@@ -1843,7 +1843,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="19">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -3042,7 +3052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="48" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>519</v>
       </c>
@@ -3696,17 +3706,17 @@
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C105">
+    <sortCondition sortBy="cellColor" ref="C2:C105" dxfId="18"/>
     <sortCondition sortBy="cellColor" ref="C2:C105" dxfId="17"/>
-    <sortCondition sortBy="cellColor" ref="C2:C105" dxfId="16"/>
   </sortState>
   <conditionalFormatting sqref="C2:C105">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3748,83 +3758,83 @@
     </row>
     <row r="2" spans="2:5" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
-        <v>210</v>
+        <v>130</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D2" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="E2" s="7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B3" s="4" t="s">
-        <v>192</v>
+        <v>128</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>108</v>
+      <c r="D3" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="E3" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="41" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="4" t="s">
-        <v>215</v>
+        <v>166</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>108</v>
+      <c r="D4" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="E4" s="7">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
-        <v>222</v>
+        <v>182</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>108</v>
+      <c r="D5" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
-        <v>120</v>
+        <v>191</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>108</v>
+      <c r="D6" s="5" t="b">
+        <v>1</v>
       </c>
       <c r="E6" s="7">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B7" s="4" t="s">
-        <v>115</v>
+        <v>210</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>108</v>
+      <c r="D7" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E7" s="7">
         <v>0.4</v>
@@ -3832,25 +3842,27 @@
     </row>
     <row r="8" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B8" s="4" t="s">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>108</v>
+      <c r="D8" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E8" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B9" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="5" t="s">
-        <v>108</v>
+        <v>215</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D9" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E9" s="7">
         <v>0.4</v>
@@ -3858,13 +3870,13 @@
     </row>
     <row r="10" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>108</v>
+      <c r="D10" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E10" s="7">
         <v>0.4</v>
@@ -3872,13 +3884,13 @@
     </row>
     <row r="11" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B11" s="4" t="s">
-        <v>226</v>
+        <v>120</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>108</v>
+      <c r="D11" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E11" s="7">
         <v>0.4</v>
@@ -3886,13 +3898,13 @@
     </row>
     <row r="12" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
-        <v>213</v>
+        <v>115</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>108</v>
+      <c r="D12" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E12" s="7">
         <v>0.4</v>
@@ -3900,27 +3912,25 @@
     </row>
     <row r="13" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>108</v>
+      <c r="D13" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E13" s="7">
-        <v>0.55000000000000004</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>108</v>
+        <v>212</v>
+      </c>
+      <c r="C14" s="4"/>
+      <c r="D14" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E14" s="7">
         <v>0.4</v>
@@ -3928,11 +3938,13 @@
     </row>
     <row r="15" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="5" t="s">
-        <v>108</v>
+        <v>207</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D15" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E15" s="7">
         <v>0.4</v>
@@ -3940,11 +3952,13 @@
     </row>
     <row r="16" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B16" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="5" t="s">
-        <v>108</v>
+        <v>226</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D16" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E16" s="7">
         <v>0.4</v>
@@ -3952,13 +3966,13 @@
     </row>
     <row r="17" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B17" s="4" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>108</v>
+      <c r="D17" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E17" s="7">
         <v>0.4</v>
@@ -3966,27 +3980,27 @@
     </row>
     <row r="18" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B18" s="4" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>108</v>
+      <c r="D18" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E18" s="7">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="19" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B19" s="4" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>108</v>
+      <c r="D19" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E19" s="7">
         <v>0.4</v>
@@ -3994,27 +4008,23 @@
     </row>
     <row r="20" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B20" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>108</v>
+        <v>224</v>
+      </c>
+      <c r="C20" s="4"/>
+      <c r="D20" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E20" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B21" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>108</v>
+        <v>219</v>
+      </c>
+      <c r="C21" s="4"/>
+      <c r="D21" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E21" s="7">
         <v>0.4</v>
@@ -4022,13 +4032,13 @@
     </row>
     <row r="22" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B22" s="4" t="s">
-        <v>121</v>
+        <v>225</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>108</v>
+        <v>502</v>
+      </c>
+      <c r="D22" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E22" s="7">
         <v>0.4</v>
@@ -4036,37 +4046,41 @@
     </row>
     <row r="23" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B23" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="5" t="s">
-        <v>108</v>
+        <v>200</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D23" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E23" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B24" s="4" t="s">
-        <v>141</v>
+        <v>195</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>108</v>
+      <c r="D24" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E24" s="7">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B25" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="C25" s="4"/>
-      <c r="D25" s="5" t="s">
-        <v>108</v>
+        <v>223</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D25" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E25" s="7">
         <v>0.4</v>
@@ -4074,25 +4088,27 @@
     </row>
     <row r="26" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B26" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C26" s="4"/>
-      <c r="D26" s="5" t="s">
-        <v>108</v>
+        <v>114</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E26" s="7">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B27" s="4" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D27" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E27" s="7">
         <v>0.4</v>
@@ -4100,37 +4116,37 @@
     </row>
     <row r="28" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B28" s="4" t="s">
-        <v>202</v>
+        <v>178</v>
       </c>
       <c r="C28" s="4"/>
-      <c r="D28" s="5" t="s">
-        <v>108</v>
+      <c r="D28" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E28" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B29" s="4" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>7</v>
+        <v>502</v>
       </c>
       <c r="D29" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" s="7">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="30" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B30" s="4" t="s">
-        <v>142</v>
+        <v>186</v>
       </c>
       <c r="C30" s="4"/>
-      <c r="D30" s="5" t="s">
-        <v>108</v>
+      <c r="D30" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E30" s="7">
         <v>0.4</v>
@@ -4138,65 +4154,63 @@
     </row>
     <row r="31" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B31" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>108</v>
+        <v>145</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E31" s="7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B32" s="4" t="s">
-        <v>177</v>
+        <v>136</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>108</v>
+      <c r="D32" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E32" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="33" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B33" s="4" t="s">
-        <v>127</v>
+        <v>202</v>
       </c>
       <c r="C33" s="4"/>
-      <c r="D33" s="5" t="s">
-        <v>108</v>
+      <c r="D33" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E33" s="7">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B34" s="4" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="C34" s="4"/>
-      <c r="D34" s="5" t="s">
-        <v>108</v>
+      <c r="D34" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E34" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="35" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B35" s="4" t="s">
-        <v>150</v>
+        <v>118</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D35" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E35" s="7">
         <v>0.4</v>
@@ -4204,81 +4218,77 @@
     </row>
     <row r="36" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B36" s="4" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>108</v>
+      <c r="D36" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E36" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B37" s="4" t="s">
-        <v>155</v>
+        <v>127</v>
       </c>
       <c r="C37" s="4"/>
-      <c r="D37" s="5" t="s">
-        <v>108</v>
+      <c r="D37" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E37" s="7">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="38" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B38" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>108</v>
+        <v>151</v>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E38" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="39" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B39" s="4" t="s">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>108</v>
+      <c r="D39" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E39" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="40" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B40" s="4" t="s">
-        <v>125</v>
+        <v>170</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>108</v>
+        <v>502</v>
+      </c>
+      <c r="D40" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E40" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="41" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B41" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>108</v>
+        <v>155</v>
+      </c>
+      <c r="C41" s="4"/>
+      <c r="D41" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E41" s="7">
         <v>0.4</v>
@@ -4286,13 +4296,13 @@
     </row>
     <row r="42" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B42" s="4" t="s">
-        <v>176</v>
+        <v>193</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>108</v>
+      <c r="D42" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E42" s="7">
         <v>0.55000000000000004</v>
@@ -4300,67 +4310,69 @@
     </row>
     <row r="43" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B43" s="4" t="s">
-        <v>217</v>
+        <v>190</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>108</v>
+      <c r="D43" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E43" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="44" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B44" s="4" t="s">
-        <v>152</v>
+        <v>125</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D44" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E44" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="45" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B45" s="4" t="s">
-        <v>220</v>
+        <v>140</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D45" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E45" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="46" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B46" s="4" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>108</v>
+      <c r="D46" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E46" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="47" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B47" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C47" s="4"/>
-      <c r="D47" s="5" t="s">
-        <v>108</v>
+        <v>217</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D47" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E47" s="7">
         <v>0.4</v>
@@ -4368,51 +4380,53 @@
     </row>
     <row r="48" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B48" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C48" s="4"/>
-      <c r="D48" s="5" t="s">
-        <v>108</v>
+        <v>152</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D48" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E48" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="49" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B49" s="4" t="s">
-        <v>174</v>
+        <v>220</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D49" s="5" t="s">
-        <v>108</v>
+      <c r="D49" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E49" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="50" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B50" s="4" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D50" s="5" t="s">
-        <v>108</v>
+      <c r="D50" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E50" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="51" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B51" s="4" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="C51" s="4"/>
-      <c r="D51" s="5" t="s">
-        <v>108</v>
+      <c r="D51" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E51" s="7">
         <v>0.4</v>
@@ -4420,51 +4434,51 @@
     </row>
     <row r="52" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B52" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>108</v>
+        <v>187</v>
+      </c>
+      <c r="C52" s="4"/>
+      <c r="D52" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E52" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="53" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B53" s="4" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D53" s="5" t="s">
-        <v>108</v>
+      <c r="D53" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E53" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="54" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B54" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C54" s="4"/>
-      <c r="D54" s="5" t="s">
-        <v>108</v>
+        <v>175</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D54" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E54" s="7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="55" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B55" s="4" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="C55" s="4"/>
-      <c r="D55" s="5" t="s">
-        <v>108</v>
+      <c r="D55" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E55" s="7">
         <v>0.4</v>
@@ -4472,39 +4486,39 @@
     </row>
     <row r="56" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B56" s="4" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D56" s="5" t="s">
-        <v>108</v>
+      <c r="D56" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E56" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="57" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B57" s="4" t="s">
-        <v>128</v>
+        <v>189</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>502</v>
       </c>
       <c r="D57" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E57" s="7">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="58" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B58" s="4" t="s">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="C58" s="4"/>
-      <c r="D58" s="5" t="s">
-        <v>108</v>
+      <c r="D58" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E58" s="7">
         <v>0.4</v>
@@ -4512,39 +4526,37 @@
     </row>
     <row r="59" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B59" s="4" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="C59" s="4"/>
-      <c r="D59" s="5" t="s">
-        <v>108</v>
+      <c r="D59" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E59" s="7">
-        <v>0.55000000000000004</v>
-      </c>
-    </row>
-    <row r="60" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B60" s="4" t="s">
-        <v>166</v>
+        <v>146</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>502</v>
       </c>
       <c r="D60" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E60" s="7">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="61" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B61" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>108</v>
+        <v>180</v>
+      </c>
+      <c r="C61" s="4"/>
+      <c r="D61" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E61" s="7">
         <v>0.4</v>
@@ -4552,211 +4564,209 @@
     </row>
     <row r="62" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B62" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C62" s="4"/>
-      <c r="D62" s="5" t="s">
-        <v>108</v>
+      <c r="D62" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E62" s="7">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="63" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B63" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="C63" s="4"/>
-      <c r="D63" s="5" t="s">
-        <v>108</v>
+        <v>124</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D63" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E63" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="64" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B64" s="4" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="C64" s="4"/>
-      <c r="D64" s="5" t="s">
-        <v>108</v>
+      <c r="D64" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E64" s="7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="65" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B65" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C65" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D65" s="5" t="s">
-        <v>108</v>
+        <v>171</v>
+      </c>
+      <c r="C65" s="4"/>
+      <c r="D65" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E65" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="66" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B66" s="4" t="s">
-        <v>157</v>
+        <v>131</v>
       </c>
       <c r="C66" s="4"/>
-      <c r="D66" s="5" t="s">
-        <v>108</v>
+      <c r="D66" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E66" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="67" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B67" s="4" t="s">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D67" s="5" t="s">
-        <v>108</v>
+        <v>502</v>
+      </c>
+      <c r="D67" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E67" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="68" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B68" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C68" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D68" s="5" t="s">
-        <v>108</v>
+        <v>157</v>
+      </c>
+      <c r="C68" s="4"/>
+      <c r="D68" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E68" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="69" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B69" s="4" t="s">
-        <v>149</v>
+        <v>181</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D69" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E69" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="70" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B70" s="4" t="s">
-        <v>143</v>
+        <v>184</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D70" s="5" t="s">
-        <v>108</v>
+      <c r="D70" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E70" s="7">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="71" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B71" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C71" s="4"/>
-      <c r="D71" s="5" t="s">
-        <v>108</v>
+        <v>149</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D71" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E71" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="72" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B72" s="4" t="s">
-        <v>182</v>
+        <v>143</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>502</v>
       </c>
       <c r="D72" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E72" s="7">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="73" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="73" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B73" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="C73" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D73" s="5" t="s">
-        <v>108</v>
+        <v>133</v>
+      </c>
+      <c r="C73" s="4"/>
+      <c r="D73" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E73" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="74" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B74" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D74" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E74" s="7">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="75" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="B75" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="C74" s="4"/>
-      <c r="D74" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E74" s="7">
+      <c r="C75" s="4"/>
+      <c r="D75" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E75" s="7">
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="75" spans="2:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="B75" s="4" t="s">
+    <row r="76" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="B76" s="4" t="s">
         <v>172</v>
-      </c>
-      <c r="C75" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D75" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E75" s="7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="76" spans="2:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="B76" s="4" t="s">
-        <v>161</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D76" s="5" t="s">
-        <v>108</v>
+      <c r="D76" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E76" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="77" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B77" s="4" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D77" s="5" t="s">
-        <v>108</v>
+      <c r="D77" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E77" s="7">
         <v>0.4</v>
@@ -4764,11 +4774,13 @@
     </row>
     <row r="78" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B78" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="C78" s="4"/>
-      <c r="D78" s="5" t="s">
-        <v>108</v>
+        <v>179</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D78" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E78" s="7">
         <v>0.4</v>
@@ -4776,13 +4788,11 @@
     </row>
     <row r="79" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B79" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>108</v>
+        <v>199</v>
+      </c>
+      <c r="C79" s="4"/>
+      <c r="D79" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E79" s="7">
         <v>0.4</v>
@@ -4790,27 +4800,27 @@
     </row>
     <row r="80" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B80" s="4" t="s">
-        <v>137</v>
+        <v>164</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D80" s="5" t="s">
-        <v>108</v>
+      <c r="D80" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E80" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="81" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B81" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D81" s="5" t="s">
-        <v>108</v>
+      <c r="D81" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E81" s="7">
         <v>0.55000000000000004</v>
@@ -4818,41 +4828,41 @@
     </row>
     <row r="82" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B82" s="4" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D82" s="5" t="s">
-        <v>108</v>
+      <c r="D82" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E82" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="83" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B83" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D83" s="5" t="s">
-        <v>108</v>
+      <c r="D83" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E83" s="7">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="84" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B84" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D84" s="5" t="s">
-        <v>108</v>
+      <c r="D84" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E84" s="7">
         <v>0.55000000000000004</v>
@@ -4860,39 +4870,39 @@
     </row>
     <row r="85" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B85" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="C85" s="4"/>
-      <c r="D85" s="5" t="s">
-        <v>108</v>
+        <v>153</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D85" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E85" s="7">
-        <v>0.4</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="86" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B86" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C86" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D86" s="5" t="s">
-        <v>108</v>
+        <v>147</v>
+      </c>
+      <c r="C86" s="4"/>
+      <c r="D86" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E86" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="87" spans="2:5" ht="32" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B87" s="4" t="s">
-        <v>126</v>
+        <v>169</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>108</v>
+        <v>502</v>
+      </c>
+      <c r="D87" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E87" s="7">
         <v>0.4</v>
@@ -4900,79 +4910,79 @@
     </row>
     <row r="88" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B88" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D88" s="5" t="s">
-        <v>108</v>
+        <v>7</v>
+      </c>
+      <c r="D88" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E88" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="89" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B89" s="4" t="s">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D89" s="5" t="s">
-        <v>108</v>
+      <c r="D89" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E89" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="90" spans="2:5" ht="48" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B90" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D90" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E90" s="7">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="91" spans="2:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="B91" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="C90" s="4"/>
-      <c r="D90" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E90" s="7">
+      <c r="C91" s="4"/>
+      <c r="D91" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E91" s="7">
         <v>0.35</v>
       </c>
     </row>
-    <row r="91" spans="2:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="B91" s="4" t="s">
+    <row r="92" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="B92" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C91" s="4" t="s">
+      <c r="C92" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D91" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E91" s="7">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="92" spans="2:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="B92" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="C92" s="4"/>
-      <c r="D92" s="5" t="s">
-        <v>108</v>
+      <c r="D92" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E92" s="7">
         <v>0.4</v>
       </c>
     </row>
-    <row r="93" spans="2:5" ht="16" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:5" ht="32" x14ac:dyDescent="0.2">
       <c r="B93" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C93" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D93" s="5" t="s">
-        <v>108</v>
+        <v>158</v>
+      </c>
+      <c r="C93" s="4"/>
+      <c r="D93" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E93" s="7">
         <v>0.4</v>
@@ -4980,11 +4990,13 @@
     </row>
     <row r="94" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B94" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C94" s="4"/>
-      <c r="D94" s="5" t="s">
-        <v>108</v>
+        <v>168</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="D94" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E94" s="7">
         <v>0.4</v>
@@ -4992,13 +5004,11 @@
     </row>
     <row r="95" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B95" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="C95" s="4" t="s">
-        <v>502</v>
-      </c>
-      <c r="D95" s="5" t="s">
-        <v>108</v>
+        <v>134</v>
+      </c>
+      <c r="C95" s="4"/>
+      <c r="D95" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E95" s="7">
         <v>0.4</v>
@@ -5006,13 +5016,13 @@
     </row>
     <row r="96" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B96" s="4" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D96" s="5" t="s">
-        <v>108</v>
+      <c r="D96" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E96" s="7">
         <v>0.4</v>
@@ -5020,16 +5030,16 @@
     </row>
     <row r="97" spans="2:5" ht="16" x14ac:dyDescent="0.2">
       <c r="B97" s="4" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>502</v>
       </c>
       <c r="D97" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" s="7">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="98" spans="2:5" ht="16" x14ac:dyDescent="0.2">
@@ -5039,8 +5049,8 @@
       <c r="C98" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D98" s="5" t="s">
-        <v>108</v>
+      <c r="D98" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E98" s="7">
         <v>0.4</v>
@@ -5053,8 +5063,8 @@
       <c r="C99" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D99" s="5" t="s">
-        <v>108</v>
+      <c r="D99" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E99" s="7">
         <v>0.4</v>
@@ -5067,8 +5077,8 @@
       <c r="C100" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D100" s="5" t="s">
-        <v>108</v>
+      <c r="D100" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E100" s="7">
         <v>0.55000000000000004</v>
@@ -5081,8 +5091,8 @@
       <c r="C101" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D101" s="5" t="s">
-        <v>108</v>
+      <c r="D101" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E101" s="7">
         <v>0.4</v>
@@ -5095,8 +5105,8 @@
       <c r="C102" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D102" s="5" t="s">
-        <v>108</v>
+      <c r="D102" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E102" s="7">
         <v>0.4</v>
@@ -5107,8 +5117,8 @@
         <v>112</v>
       </c>
       <c r="C103" s="4"/>
-      <c r="D103" s="5" t="s">
-        <v>108</v>
+      <c r="D103" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E103" s="7">
         <v>0.55000000000000004</v>
@@ -5121,8 +5131,8 @@
       <c r="C104" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D104" s="5" t="s">
-        <v>108</v>
+      <c r="D104" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E104" s="7">
         <v>0.4</v>
@@ -5135,8 +5145,8 @@
       <c r="C105" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D105" s="5" t="s">
-        <v>108</v>
+      <c r="D105" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E105" s="7">
         <v>0.4</v>
@@ -5147,8 +5157,8 @@
         <v>228</v>
       </c>
       <c r="C106" s="4"/>
-      <c r="D106" s="5" t="s">
-        <v>108</v>
+      <c r="D106" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E106" s="7">
         <v>0.55000000000000004</v>
@@ -5161,8 +5171,8 @@
       <c r="C107" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D107" s="5" t="s">
-        <v>108</v>
+      <c r="D107" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E107" s="7">
         <v>0.55000000000000004</v>
@@ -5175,8 +5185,8 @@
       <c r="C108" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D108" s="5" t="s">
-        <v>108</v>
+      <c r="D108" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E108" s="7">
         <v>0.4</v>
@@ -5189,8 +5199,8 @@
       <c r="C109" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D109" s="5" t="s">
-        <v>108</v>
+      <c r="D109" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E109" s="7">
         <v>0.4</v>
@@ -5203,8 +5213,8 @@
       <c r="C110" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D110" s="5" t="s">
-        <v>108</v>
+      <c r="D110" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E110" s="7">
         <v>0.4</v>
@@ -5217,8 +5227,8 @@
       <c r="C111" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D111" s="5" t="s">
-        <v>108</v>
+      <c r="D111" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E111" s="7">
         <v>0.4</v>
@@ -5231,8 +5241,8 @@
       <c r="C112" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D112" s="5" t="s">
-        <v>108</v>
+      <c r="D112" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E112" s="7">
         <v>0.4</v>
@@ -5243,8 +5253,8 @@
         <v>113</v>
       </c>
       <c r="C113" s="4"/>
-      <c r="D113" s="5" t="s">
-        <v>108</v>
+      <c r="D113" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E113" s="7">
         <v>0.4</v>
@@ -5255,8 +5265,8 @@
         <v>206</v>
       </c>
       <c r="C114" s="4"/>
-      <c r="D114" s="5" t="s">
-        <v>108</v>
+      <c r="D114" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E114" s="7">
         <v>0.4</v>
@@ -5269,8 +5279,8 @@
       <c r="C115" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D115" s="5" t="s">
-        <v>108</v>
+      <c r="D115" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E115" s="7">
         <v>0.4</v>
@@ -5283,8 +5293,8 @@
       <c r="C116" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D116" s="5" t="s">
-        <v>108</v>
+      <c r="D116" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E116" s="7">
         <v>0.55000000000000004</v>
@@ -5297,8 +5307,8 @@
       <c r="C117" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D117" s="5" t="s">
-        <v>108</v>
+      <c r="D117" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E117" s="7">
         <v>0.4</v>
@@ -5311,8 +5321,8 @@
       <c r="C118" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D118" s="5" t="s">
-        <v>108</v>
+      <c r="D118" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E118" s="7">
         <v>0.4</v>
@@ -5325,8 +5335,8 @@
       <c r="C119" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D119" s="5" t="s">
-        <v>108</v>
+      <c r="D119" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E119" s="7">
         <v>0.4</v>
@@ -5339,8 +5349,8 @@
       <c r="C120" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D120" s="5" t="s">
-        <v>108</v>
+      <c r="D120" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E120" s="7">
         <v>0.4</v>
@@ -5353,8 +5363,8 @@
       <c r="C121" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="D121" s="5" t="s">
-        <v>108</v>
+      <c r="D121" s="5" t="b">
+        <v>0</v>
       </c>
       <c r="E121" s="7">
         <v>0.4</v>
@@ -5362,16 +5372,21 @@
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:E121">
-    <sortCondition ref="B2:B121"/>
+    <sortCondition descending="1" ref="D2:D121"/>
   </sortState>
   <conditionalFormatting sqref="C2:C88">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D122">
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
       <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:D121">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -6877,32 +6892,32 @@
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D85">
-    <sortCondition sortBy="cellColor" ref="C2:C85" dxfId="15"/>
+    <sortCondition sortBy="cellColor" ref="C2:C85" dxfId="16"/>
+    <sortCondition descending="1" sortBy="cellColor" ref="C2:C85" dxfId="15"/>
     <sortCondition descending="1" sortBy="cellColor" ref="C2:C85" dxfId="14"/>
-    <sortCondition descending="1" sortBy="cellColor" ref="C2:C85" dxfId="13"/>
   </sortState>
   <conditionalFormatting sqref="C31:D31 D31:D85">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C31:D88 C2:E30">
-    <cfRule type="cellIs" dxfId="6" priority="63" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="63" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C61:D85">
-    <cfRule type="cellIs" dxfId="5" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="15" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:E30 C32:D60 C76:D82">
-    <cfRule type="cellIs" dxfId="4" priority="29" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="29" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D29">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7732,7 +7747,7 @@
     <sortCondition ref="B2:B37"/>
   </sortState>
   <conditionalFormatting sqref="C2:C88">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8344,7 +8359,7 @@
     <sortCondition ref="B2:B24"/>
   </sortState>
   <conditionalFormatting sqref="C2:C88">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9631,7 +9646,7 @@
     <sortCondition ref="B2:B99"/>
   </sortState>
   <conditionalFormatting sqref="C2:C88">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"Maybe"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>